<commit_message>
Review text no longer mandatory
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta.xlsx
+++ b/docs/Työajan seuranta.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arttu\Dropbox\Koulu\Web-ohjelmoinnin sovellusprojekti\Movieproject\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A46581E-66D9-4D3D-A45C-42C953849AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58844D71-5040-46A8-B22B-5AFB99C23D3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15300" yWindow="4830" windowWidth="17685" windowHeight="14025" activeTab="2" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
+    <workbookView xWindow="3345" yWindow="5955" windowWidth="17670" windowHeight="9870" activeTab="2" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
   <sheets>
     <sheet name="Laura Similä" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="35">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -149,6 +149,12 @@
   </si>
   <si>
     <t>APIn korjailua</t>
+  </si>
+  <si>
+    <t>22.9.</t>
+  </si>
+  <si>
+    <t>Review API create &amp; search</t>
   </si>
 </sst>
 </file>
@@ -704,7 +710,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
@@ -773,6 +779,17 @@
       </c>
       <c r="C6">
         <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>33</v>
+      </c>
+      <c r="B7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C7">
+        <v>3.5</v>
       </c>
     </row>
   </sheetData>
@@ -821,20 +838,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1018,19 +1035,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
update tracking of working hours
</commit_message>
<xml_diff>
--- a/docs/Työajan seuranta.xlsx
+++ b/docs/Työajan seuranta.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30516"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unioulu-my.sharepoint.com/personal/lsimila24_students_oamk_fi/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bb667e905e7871ab/Documents/Git/movieproject/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{647DC8A6-F150-4022-807D-2169B52DC997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="8_{647DC8A6-F150-4022-807D-2169B52DC997}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1AC3380-0BB0-4A0E-8B41-1E0F440B918F}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6120" windowWidth="29040" windowHeight="15720" xr2:uid="{B7036960-D674-4B76-B564-D076AACD5E6B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="40">
   <si>
     <t>Ryhmä:</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Aika</t>
-  </si>
-  <si>
-    <t>PR Reviews käytetty aika (projektin aikana) ~ 5 h</t>
   </si>
   <si>
     <t>7.9.</t>
@@ -132,12 +129,63 @@
   <si>
     <t>2.5 h</t>
   </si>
+  <si>
+    <t>19.9.</t>
+  </si>
+  <si>
+    <t>20.9.</t>
+  </si>
+  <si>
+    <t>Seuraavan sprintin suunnittelu
+Backendin GitHub Actions CI:n suunnittelu
+Automatisoidun backend-testisuiten liittäminen CI-workflow'hun
+Palaveria</t>
+  </si>
+  <si>
+    <t>3h</t>
+  </si>
+  <si>
+    <t>21.9.</t>
+  </si>
+  <si>
+    <t>Palaveria</t>
+  </si>
+  <si>
+    <t>0.75h</t>
+  </si>
+  <si>
+    <t>23.9.</t>
+  </si>
+  <si>
+    <t>Review- ja Favorites-tietokantatehtävien tilanteen tarkistus suhteessa nykyiseen tietokantaskeemaan</t>
+  </si>
+  <si>
+    <t>0.5h</t>
+  </si>
+  <si>
+    <t>24.9.</t>
+  </si>
+  <si>
+    <t>Favorite Movies Management -toiminnallisuuden suunnittelu
+Favorites-backendin toteutus
+Favorites-backendin toteutus
+Favorite Movies List -sivun toteutus
+Favorites-toiminnallisuuden integrointi profiiliin
+Favorites-UI:n viimeistely
+Korjauksia ja bugitiketin teko</t>
+  </si>
+  <si>
+    <t>5.5h</t>
+  </si>
+  <si>
+    <t>PR Reviews käytetty aika (projektin aikana) ~ 6.25 h</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -166,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -180,6 +228,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -198,10 +249,14 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022 -teema">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -239,7 +294,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -345,7 +400,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -487,7 +542,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -495,17 +550,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BD4D073-EB2D-44A2-86BF-660E3721AF80}">
-  <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
     <col min="2" max="2" width="93.7109375" customWidth="1"/>
     <col min="3" max="4" width="13.28515625" customWidth="1"/>
-    <col min="5" max="5" width="43.140625" customWidth="1"/>
+    <col min="5" max="5" width="45.7109375" customWidth="1"/>
     <col min="6" max="6" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -516,7 +571,7 @@
       <c r="D1" s="3"/>
       <c r="E1" s="3"/>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
@@ -528,112 +583,156 @@
       </c>
       <c r="D2" s="3"/>
       <c r="E2" s="3" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="28.5" customHeight="1">
-      <c r="A3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="3" t="s">
         <v>6</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>7</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
     </row>
-    <row r="4" spans="1:5" ht="60.75">
+    <row r="4" spans="1:5" ht="60" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
       </c>
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
     </row>
-    <row r="5" spans="1:5" ht="30.75">
+    <row r="5" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="3" t="s">
         <v>12</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>13</v>
       </c>
       <c r="D5" s="3"/>
       <c r="E5" s="3"/>
     </row>
-    <row r="6" spans="1:5" ht="45.75">
+    <row r="6" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="5" t="s">
-        <v>15</v>
-      </c>
       <c r="C6" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="D7" s="3"/>
       <c r="E7" s="3"/>
     </row>
-    <row r="8" spans="1:5" ht="45.75">
+    <row r="8" spans="1:5" ht="45" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>21</v>
       </c>
       <c r="D8" s="3"/>
       <c r="E8" s="3"/>
     </row>
-    <row r="9" spans="1:5" ht="30.75">
+    <row r="9" spans="1:5" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="D9" s="3"/>
       <c r="E9" s="3"/>
     </row>
-    <row r="10" spans="1:5" ht="30.75">
-      <c r="A10" s="3">
-        <v>19.899999999999999</v>
+    <row r="10" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>25</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>26</v>
       </c>
       <c r="D10" s="3"/>
       <c r="E10" s="3"/>
+    </row>
+    <row r="11" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="105" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>38</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -643,14 +742,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCCA3CA-2A17-42EC-86E5-CF5FE2A8D439}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.140625" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" customWidth="1"/>
     <col min="3" max="3" width="11.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -658,7 +757,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -669,13 +768,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
   </sheetData>
@@ -686,14 +785,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C1EECD9-4AD3-41AF-8923-B28678799497}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.85546875" customWidth="1"/>
     <col min="2" max="2" width="31.42578125" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -701,7 +800,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -712,13 +811,13 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
     </row>
   </sheetData>
@@ -729,14 +828,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{74BC3D70-9A8B-4A59-8343-1D3356DFB267}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.85546875" customWidth="1"/>
     <col min="2" max="2" width="30.85546875" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -744,7 +843,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -755,10 +854,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1"/>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
     </row>
   </sheetData>
@@ -767,6 +866,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009BAF6AFB37B6774A9122C6036818BC92" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c611cd0fe7e35dfe638a44e659100205">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="44038759-07ae-40d4-bc3d-7c9fb0b3775b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="36a43d4c38ea7f7b42b5de64d2c1c906" ns3:_="">
     <xsd:import namespace="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
@@ -946,33 +1062,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="44038759-07ae-40d4-bc3d-7c9fb0b3775b" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{28C42445-4535-4827-89B5-92D7D04A90E8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D3DBD177-6275-4D31-B82C-61F9284D9B7B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B52374CD-1656-483C-BC7A-A879F7105755}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="44038759-07ae-40d4-bc3d-7c9fb0b3775b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>